<commit_message>
added python invoice generator and updated files
</commit_message>
<xml_diff>
--- a/backend/RAHUL_SERVICES_INVOICE.xlsx
+++ b/backend/RAHUL_SERVICES_INVOICE.xlsx
@@ -462,7 +462,7 @@
     <row r="4">
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>RAHUL SERVICE</t>
+          <t>ACME PVT LTD</t>
         </is>
       </c>
       <c r="C4" s="2" t="n"/>
@@ -492,7 +492,7 @@
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>GST NO : Laudantium iure qui   Phone No: +1 (914) 454-1211</t>
+          <t>GST NO : Eaque pariatur Volu   Phone No: +1 (806) 696-6555</t>
         </is>
       </c>
       <c r="C6" s="2" t="n"/>
@@ -501,7 +501,7 @@
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>DATE: 1973-11-06</t>
+          <t>DATE: 2009-07-09</t>
         </is>
       </c>
       <c r="H6" s="2" t="n"/>
@@ -511,7 +511,7 @@
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>INVOICE NO: INV/2026/0002</t>
+          <t xml:space="preserve">INVOICE NO: </t>
         </is>
       </c>
       <c r="C7" s="2" t="n"/>
@@ -520,7 +520,7 @@
       <c r="F7" s="2" t="n"/>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>TRANSPORT BY : Do qui ipsum minim i</t>
+          <t>TRANSPORT BY : Culpa et fugiat fac</t>
         </is>
       </c>
       <c r="H7" s="2" t="n"/>
@@ -530,7 +530,7 @@
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>REVERSE CHARGE: Asperiores saepe cul</t>
+          <t xml:space="preserve">REVERSE CHARGE: Non est provident </t>
         </is>
       </c>
       <c r="C8" s="2" t="n"/>
@@ -539,7 +539,7 @@
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>VEHICLE NO: Lorem libero iure ma</t>
+          <t>VEHICLE NO: Magni dolor inventor</t>
         </is>
       </c>
       <c r="H8" s="2" t="n"/>
@@ -549,7 +549,7 @@
     <row r="9">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>INVOICE DATE: 1973-11-06</t>
+          <t>INVOICE DATE: 2009-07-09</t>
         </is>
       </c>
       <c r="C9" s="2" t="n"/>
@@ -558,7 +558,7 @@
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>DATE OF DELIVERY: 1992-11-04</t>
+          <t>DATE OF DELIVERY: 2008-12-05</t>
         </is>
       </c>
       <c r="H9" s="2" t="n"/>
@@ -568,7 +568,7 @@
     <row r="10">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>STATE : Linda Arnold   STATE CODE : Labore non fugiat si</t>
+          <t>STATE : Danielle Willis   STATE CODE : Sapiente perferendis</t>
         </is>
       </c>
       <c r="C10" s="2" t="n"/>
@@ -577,7 +577,7 @@
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>PLACE OF DELIVERY: Excepteur voluptatem</t>
+          <t>PLACE OF DELIVERY: Praesentium corporis</t>
         </is>
       </c>
       <c r="H10" s="2" t="n"/>
@@ -613,7 +613,7 @@
     <row r="13">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>NAME : Andrew Levine</t>
+          <t>NAME : Clare Shields</t>
         </is>
       </c>
       <c r="C13" s="2" t="n"/>
@@ -632,7 +632,7 @@
     <row r="14">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>TR NO : Optio inventore qua</t>
+          <t>TR NO : Aut impedit velit d</t>
         </is>
       </c>
       <c r="C14" s="2" t="n"/>
@@ -641,7 +641,7 @@
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>NAME: Duncan Finch</t>
+          <t>NAME: Eric Barr</t>
         </is>
       </c>
       <c r="H14" s="2" t="n"/>
@@ -651,7 +651,7 @@
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADDRESS : Laborum Quas dolor </t>
+          <t>ADDRESS : Odit reprehenderit q</t>
         </is>
       </c>
       <c r="C15" s="2" t="n"/>
@@ -660,7 +660,7 @@
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>ADDRESS: Non officia facere d</t>
+          <t>ADDRESS: Itaque nisi ipsa co</t>
         </is>
       </c>
       <c r="H15" s="2" t="n"/>
@@ -670,7 +670,7 @@
     <row r="16">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>GST NO : Non omnis ea volupta   STATE CODE : Deserunt in exceptur</t>
+          <t>GST NO : Earum magni inventor   STATE CODE : In eos quisquam dele</t>
         </is>
       </c>
       <c r="C16" s="2" t="n"/>
@@ -679,7 +679,7 @@
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>GST NO : Est doloremque at a   STATE CODE : Sed optio sed conse</t>
+          <t>GST NO : Nihil voluptates est   STATE CODE : Nam provident conse</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
@@ -750,39 +750,39 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Qui voluptatem nemo </t>
+          <t>Laudantium odio ame</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Nihil distinctio Al</t>
+          <t>Quas ipsa voluptatu</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>25.0 nos.</t>
+          <t>48.0 nos.</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>79</v>
+        <v>120</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>1975</v>
+        <v>5760</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>177.75</v>
+        <v>518.4</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>177.75</v>
+        <v>518.4</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>2330.5</v>
+        <v>6796.8</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Fuga Laborum corrup</t>
+          <t>Fuga Adipisci conse</t>
         </is>
       </c>
       <c r="C20" s="2" t="n"/>
@@ -808,7 +808,7 @@
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="n"/>
       <c r="J21" s="2" t="n">
-        <v>2330.5</v>
+        <v>6796.8</v>
       </c>
     </row>
     <row r="22">
@@ -829,7 +829,7 @@
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>RUPEES-TWO-THOUSAND-TWO-HUNDRED-NINETY-EIGHT ONLY.</t>
+          <t>RUPEES-SIX-THOUSAND-SEVEN-HUNDRED-TWENTY-SEVEN ONLY.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n"/>
@@ -855,7 +855,7 @@
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="n">
-        <v>33</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25">
@@ -872,7 +872,7 @@
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="n"/>
       <c r="J25" s="2" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="26">
@@ -889,7 +889,7 @@
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="n"/>
       <c r="J26" s="2" t="n">
-        <v>2298</v>
+        <v>6727</v>
       </c>
     </row>
     <row r="27">
@@ -906,7 +906,7 @@
     <row r="28">
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>FOR RAHUL SERVICE</t>
+          <t>FOR ACME PVT LTD</t>
         </is>
       </c>
       <c r="C28" s="2" t="n"/>

</xml_diff>